<commit_message>
v3.3: chore - aoi_tt & aoi_rs decoration
</commit_message>
<xml_diff>
--- a/resources/spc_sheet_oos_decoration.xlsx
+++ b/resources/spc_sheet_oos_decoration.xlsx
@@ -10892,7 +10892,7 @@
         <v>-7.6155</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01529912280701755</v>
+        <v>0.01529912280701754</v>
       </c>
       <c r="J3" t="n">
         <v>6.5</v>
@@ -11210,7 +11210,7 @@
         <v>-3.4499</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.04229736842105266</v>
+        <v>-0.04229736842105263</v>
       </c>
       <c r="J9" t="n">
         <v>6.5</v>
@@ -11899,7 +11899,7 @@
         <v>-6.8108</v>
       </c>
       <c r="I22" t="n">
-        <v>-0.07766140350877195</v>
+        <v>-0.07766140350877193</v>
       </c>
       <c r="J22" t="n">
         <v>6.5</v>
@@ -12058,7 +12058,7 @@
         <v>-4.1055</v>
       </c>
       <c r="I25" t="n">
-        <v>0.4946271929824562</v>
+        <v>0.4946271929824561</v>
       </c>
       <c r="J25" t="n">
         <v>6.5</v>
@@ -12482,7 +12482,7 @@
         <v>-6.2914</v>
       </c>
       <c r="I33" t="n">
-        <v>0.03470701754385964</v>
+        <v>0.03470701754385961</v>
       </c>
       <c r="J33" t="n">
         <v>6.5</v>
@@ -12535,7 +12535,7 @@
         <v>-5.1599</v>
       </c>
       <c r="I34" t="n">
-        <v>-0.4605105263157895</v>
+        <v>-0.4605105263157894</v>
       </c>
       <c r="J34" t="n">
         <v>6.5</v>
@@ -13118,7 +13118,7 @@
         <v>-4.4651</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.04652807017543856</v>
+        <v>-0.04652807017543861</v>
       </c>
       <c r="J45" t="n">
         <v>6.5</v>
@@ -13277,7 +13277,7 @@
         <v>-5.8719</v>
       </c>
       <c r="I48" t="n">
-        <v>0.3151008771929824</v>
+        <v>0.3151008771929825</v>
       </c>
       <c r="J48" t="n">
         <v>6.5</v>
@@ -13542,7 +13542,7 @@
         <v>-8.343400000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.8040798245614035</v>
+        <v>-0.8040798245614036</v>
       </c>
       <c r="J53" t="n">
         <v>6.5</v>
@@ -13860,7 +13860,7 @@
         <v>-6.9804</v>
       </c>
       <c r="I59" t="n">
-        <v>-0.008550000000000026</v>
+        <v>-0.008550000000000058</v>
       </c>
       <c r="J59" t="n">
         <v>6.5</v>
@@ -14549,7 +14549,7 @@
         <v>-4.5534</v>
       </c>
       <c r="I72" t="n">
-        <v>0.6093447368421052</v>
+        <v>0.6093447368421053</v>
       </c>
       <c r="J72" t="n">
         <v>6.5</v>
@@ -14708,7 +14708,7 @@
         <v>-5.7729</v>
       </c>
       <c r="I75" t="n">
-        <v>0.2905122807017543</v>
+        <v>0.2905122807017544</v>
       </c>
       <c r="J75" t="n">
         <v>6.5</v>
@@ -14814,7 +14814,7 @@
         <v>-4.8514</v>
       </c>
       <c r="I77" t="n">
-        <v>1.477787719298246</v>
+        <v>1.477787719298245</v>
       </c>
       <c r="J77" t="n">
         <v>6.5</v>
@@ -14973,7 +14973,7 @@
         <v>-5.8919</v>
       </c>
       <c r="I80" t="n">
-        <v>-0.006774561403508777</v>
+        <v>-0.006774561403508803</v>
       </c>
       <c r="J80" t="n">
         <v>6.5</v>
@@ -15079,7 +15079,7 @@
         <v>-5.2636</v>
       </c>
       <c r="I82" t="n">
-        <v>-0.09407280701754382</v>
+        <v>-0.09407280701754384</v>
       </c>
       <c r="J82" t="n">
         <v>6.5</v>
@@ -15397,7 +15397,7 @@
         <v>-6.3484</v>
       </c>
       <c r="I88" t="n">
-        <v>0.09611228070175443</v>
+        <v>0.0961122807017544</v>
       </c>
       <c r="J88" t="n">
         <v>6.5</v>
@@ -15874,7 +15874,7 @@
         <v>-6.9829</v>
       </c>
       <c r="I97" t="n">
-        <v>-0.6455096491228069</v>
+        <v>-0.6455096491228072</v>
       </c>
       <c r="J97" t="n">
         <v>6.5</v>
@@ -16351,7 +16351,7 @@
         <v>-4.4856</v>
       </c>
       <c r="I106" t="n">
-        <v>0.496932456140351</v>
+        <v>0.4969324561403509</v>
       </c>
       <c r="J106" t="n">
         <v>6.5</v>
@@ -16775,7 +16775,7 @@
         <v>-8.3277</v>
       </c>
       <c r="I114" t="n">
-        <v>-0.9198491228070176</v>
+        <v>-0.9198491228070175</v>
       </c>
       <c r="J114" t="n">
         <v>6.5</v>
@@ -16934,7 +16934,7 @@
         <v>-4.0971</v>
       </c>
       <c r="I117" t="n">
-        <v>0.5978482456140352</v>
+        <v>0.597848245614035</v>
       </c>
       <c r="J117" t="n">
         <v>6.5</v>
@@ -17040,7 +17040,7 @@
         <v>-5.0645</v>
       </c>
       <c r="I119" t="n">
-        <v>0.03353596491228069</v>
+        <v>0.03353596491228068</v>
       </c>
       <c r="J119" t="n">
         <v>6.5</v>
@@ -17252,7 +17252,7 @@
         <v>-6.1071</v>
       </c>
       <c r="I123" t="n">
-        <v>0.06978508771929821</v>
+        <v>0.06978508771929823</v>
       </c>
       <c r="J123" t="n">
         <v>6.5</v>
@@ -17782,7 +17782,7 @@
         <v>-4.3932</v>
       </c>
       <c r="I133" t="n">
-        <v>0.8818175438596491</v>
+        <v>0.8818175438596492</v>
       </c>
       <c r="J133" t="n">
         <v>6.5</v>
@@ -18577,7 +18577,7 @@
         <v>-6.718</v>
       </c>
       <c r="I148" t="n">
-        <v>0.5547491228070176</v>
+        <v>0.5547491228070175</v>
       </c>
       <c r="J148" t="n">
         <v>6.5</v>
@@ -18736,7 +18736,7 @@
         <v>-5.6271</v>
       </c>
       <c r="I151" t="n">
-        <v>0.8492342105263158</v>
+        <v>0.8492342105263159</v>
       </c>
       <c r="J151" t="n">
         <v>6.5</v>
@@ -19001,7 +19001,7 @@
         <v>-25.5842</v>
       </c>
       <c r="I156" t="n">
-        <v>0.9268140350877192</v>
+        <v>0.9268140350877193</v>
       </c>
       <c r="J156" t="n">
         <v>6.5</v>
@@ -19213,7 +19213,7 @@
         <v>-6.347</v>
       </c>
       <c r="I160" t="n">
-        <v>0.9459850877192983</v>
+        <v>0.9459850877192982</v>
       </c>
       <c r="J160" t="n">
         <v>6.5</v>
@@ -19531,7 +19531,7 @@
         <v>-5.6733</v>
       </c>
       <c r="I166" t="n">
-        <v>-0.1435087719298246</v>
+        <v>-0.1435087719298245</v>
       </c>
       <c r="J166" t="n">
         <v>6.5</v>
@@ -20167,7 +20167,7 @@
         <v>-14.0222</v>
       </c>
       <c r="I178" t="n">
-        <v>0.8890823008849558</v>
+        <v>0.8890823008849557</v>
       </c>
       <c r="J178" t="n">
         <v>6.5</v>
@@ -20909,7 +20909,7 @@
         <v>-7.7786</v>
       </c>
       <c r="I192" t="n">
-        <v>-0.3039491228070175</v>
+        <v>-0.3039491228070176</v>
       </c>
       <c r="J192" t="n">
         <v>6.5</v>
@@ -21280,7 +21280,7 @@
         <v>-6.6293</v>
       </c>
       <c r="I199" t="n">
-        <v>0.9794122807017543</v>
+        <v>0.9794122807017545</v>
       </c>
       <c r="J199" t="n">
         <v>6.5</v>
@@ -21916,7 +21916,7 @@
         <v>-7.2617</v>
       </c>
       <c r="I211" t="n">
-        <v>-0.005909649122807063</v>
+        <v>-0.00590964912280703</v>
       </c>
       <c r="J211" t="n">
         <v>6.5</v>
@@ -22075,7 +22075,7 @@
         <v>-7.7634</v>
       </c>
       <c r="I214" t="n">
-        <v>-0.07643596491228072</v>
+        <v>-0.07643596491228073</v>
       </c>
       <c r="J214" t="n">
         <v>6.5</v>
@@ -23400,7 +23400,7 @@
         <v>-6.5046</v>
       </c>
       <c r="I239" t="n">
-        <v>0.7791377192982457</v>
+        <v>0.7791377192982456</v>
       </c>
       <c r="J239" t="n">
         <v>6.5</v>
@@ -23771,7 +23771,7 @@
         <v>-4.9538</v>
       </c>
       <c r="I246" t="n">
-        <v>0.614871052631579</v>
+        <v>0.6148710526315789</v>
       </c>
       <c r="J246" t="n">
         <v>6.5</v>
@@ -23983,7 +23983,7 @@
         <v>-6.1278</v>
       </c>
       <c r="I250" t="n">
-        <v>-0.0579815789473684</v>
+        <v>-0.05798157894736843</v>
       </c>
       <c r="J250" t="n">
         <v>6.5</v>
@@ -25149,7 +25149,7 @@
         <v>-5.5515</v>
       </c>
       <c r="I272" t="n">
-        <v>0.3501815789473685</v>
+        <v>0.3501815789473684</v>
       </c>
       <c r="J272" t="n">
         <v>6.5</v>
@@ -25202,7 +25202,7 @@
         <v>-6.2885</v>
       </c>
       <c r="I273" t="n">
-        <v>0.04088859649122807</v>
+        <v>0.04088859649122806</v>
       </c>
       <c r="J273" t="n">
         <v>6.5</v>
@@ -25308,7 +25308,7 @@
         <v>-6.532</v>
       </c>
       <c r="I275" t="n">
-        <v>0.01685877192982452</v>
+        <v>0.01685877192982455</v>
       </c>
       <c r="J275" t="n">
         <v>6.5</v>
@@ -25361,7 +25361,7 @@
         <v>-8.580500000000001</v>
       </c>
       <c r="I276" t="n">
-        <v>-0.4958578947368421</v>
+        <v>-0.4958578947368422</v>
       </c>
       <c r="J276" t="n">
         <v>6.5</v>
@@ -25520,7 +25520,7 @@
         <v>-6.6815</v>
       </c>
       <c r="I279" t="n">
-        <v>0.3845070175438596</v>
+        <v>0.3845070175438597</v>
       </c>
       <c r="J279" t="n">
         <v>6.5</v>
@@ -26103,7 +26103,7 @@
         <v>-6.1323</v>
       </c>
       <c r="I290" t="n">
-        <v>-0.2874561403508771</v>
+        <v>-0.2874561403508772</v>
       </c>
       <c r="J290" t="n">
         <v>6.5</v>
@@ -26209,7 +26209,7 @@
         <v>-3.3104</v>
       </c>
       <c r="I292" t="n">
-        <v>0.8435719298245615</v>
+        <v>0.8435719298245613</v>
       </c>
       <c r="J292" t="n">
         <v>6.5</v>
@@ -26527,7 +26527,7 @@
         <v>-6.2062</v>
       </c>
       <c r="I298" t="n">
-        <v>0.3236368421052631</v>
+        <v>0.3236368421052632</v>
       </c>
       <c r="J298" t="n">
         <v>6.5</v>
@@ -26633,7 +26633,7 @@
         <v>-4.3444</v>
       </c>
       <c r="I300" t="n">
-        <v>0.6657157894736841</v>
+        <v>0.6657157894736843</v>
       </c>
       <c r="J300" t="n">
         <v>6.5</v>
@@ -28011,7 +28011,7 @@
         <v>-6.5794</v>
       </c>
       <c r="I326" t="n">
-        <v>0.4163964912280703</v>
+        <v>0.4163964912280702</v>
       </c>
       <c r="J326" t="n">
         <v>6.5</v>
@@ -29389,7 +29389,7 @@
         <v>-6.3705</v>
       </c>
       <c r="I352" t="n">
-        <v>0.09694385964912278</v>
+        <v>0.09694385964912279</v>
       </c>
       <c r="J352" t="n">
         <v>6.5</v>
@@ -31085,7 +31085,7 @@
         <v>-5.9691</v>
       </c>
       <c r="I384" t="n">
-        <v>-0.09673684210526313</v>
+        <v>-0.09673684210526315</v>
       </c>
       <c r="J384" t="n">
         <v>6.5</v>
@@ -31933,7 +31933,7 @@
         <v>-7.181</v>
       </c>
       <c r="I400" t="n">
-        <v>0.2636938596491228</v>
+        <v>0.2636938596491227</v>
       </c>
       <c r="J400" t="n">
         <v>6.5</v>
@@ -34053,7 +34053,7 @@
         <v>-8.6503</v>
       </c>
       <c r="I440" t="n">
-        <v>0.04960877192982458</v>
+        <v>0.04960877192982456</v>
       </c>
       <c r="J440" t="n">
         <v>6.5</v>
@@ -34318,7 +34318,7 @@
         <v>-7.706</v>
       </c>
       <c r="I445" t="n">
-        <v>-0.01646666666666669</v>
+        <v>-0.0164666666666667</v>
       </c>
       <c r="J445" t="n">
         <v>6.5</v>
@@ -34795,7 +34795,7 @@
         <v>-7.3081</v>
       </c>
       <c r="I454" t="n">
-        <v>0.06260964912280706</v>
+        <v>0.06260964912280703</v>
       </c>
       <c r="J454" t="n">
         <v>6.5</v>
@@ -34901,7 +34901,7 @@
         <v>-5.8034</v>
       </c>
       <c r="I456" t="n">
-        <v>0.01259649122807016</v>
+        <v>0.01259649122807015</v>
       </c>
       <c r="J456" t="n">
         <v>6.5</v>
@@ -35537,7 +35537,7 @@
         <v>-6.4277</v>
       </c>
       <c r="I468" t="n">
-        <v>0.562111403508772</v>
+        <v>0.5621114035087719</v>
       </c>
       <c r="J468" t="n">
         <v>6.5</v>

</xml_diff>